<commit_message>
Add job applications and shortlist for 2026-10-15
</commit_message>
<xml_diff>
--- a/Job_Applications_Tracker.xlsx
+++ b/Job_Applications_Tracker.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -910,6 +910,1162 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Deservely Technologies</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Developer (Claude AI-Powered)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4477503300/</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Resume_FullStackAI_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Claude/AI dev; matches Anthropic/RAG exp; 'Senior' slight stretch; verify JD</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Smart Energy Water</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4478125060/</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>energy-SaaS product co; clean full-stack fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>VOICE OF HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Backend Developer - AI &amp; Automation</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Gurugram</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4478858013/</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Resume_FullStackAI_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>AI/automation backend; NOT same as Voiceoc Innovations - confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Concentrix</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4478036422/</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Resume_NodeReact_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>large CX firm remote; verify JD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Appinventiv</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4476088845/</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Resume_NodeReact_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>dev agency; verify stack (MERN/RN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Weekday AI (YC W21)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Gurugram</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4479270124/</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Resume_NodeJS_TechQware.pdf</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>hiring marketplace - role for a client; verify Node</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Brandlio</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4478403789/</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Resume_NodeReact_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>remote startup; verify JD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Javascript Developer</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4477157147/</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Resume_SWE_NIIT.pdf</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>large MNC; verify stack</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Data Eminence</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Web Developer</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4478451828/</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Resume_Frontend.pdf</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>generic web dev; low signal; verify JD</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Frontend Engineer - Earn</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4476258189/</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Resume_Frontend.pdf</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>aggregator; real employer hidden; 'Earn' may be fintech/crypto; verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Crossing Hurdles</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Software Engineer (Remote)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4478411616/</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Resume_FullStackAI_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>contract $50-100/hr; likely US hours; verify terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Moneymul Technologies</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Delhi/NCR, Noida</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-senior-full-stack-developer-moneymul-technologies-pvt-ltd-noida-delhi-ncr-3-to-8-years-060826010956</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>BULLSEYE Node/React/TS/Postgres/Sequelize/Prisma; 3-8y; tailor resume recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Concrete Software Solutions</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Node/React/REST/CI-CD; 2-4y; link not captured - search Naukri</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Acrapath</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Full Stack Developer (ReactNative)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>New Delhi (Kirti Nagar)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-full-stack-developer-reactnative-acrapath-new-delhi-1-to-4-years-121026007841</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Node/ReactNative/Express/Redux; 4.25-5.5 LPA below 8 ask</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tenacious Hr Solution</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Delhi/NCR, Bengaluru, Mumbai</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>consultant; 6-16 LPA; React/Node + Java/Angular; link not captured - search</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Maivita</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-full-stack-developer-maivita-noida-0-to-3-years-151026019640</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>MERN; 0-3y + 2.5-5 LPA; lower priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ARM Infotech</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-full-stack-developer-arm-infotech-noida-3-to-5-years-141026915316</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Java-heavy + JS/Postgres/Mongo; 3-5y; medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ProVal Tech</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sr Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-sr-full-stack-developer-proval-technologies-noida-3-to-7-years-141026506793</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Resume_FullStackAI_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>JS serverless Deno/Edge + AI tooling; 2.4-star check culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Protiviti India</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Full Stack Developer (Entrust)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Resume_NodeReact_Remote.pdf</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>vague stack; UK shift; link not captured - search</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Edge (EDGE Executive Search)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Java Full Stack Developer - React</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Gurugram, Delhi/NCR</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Resume_MERN.pdf</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Java/Spring primary + React; 3-5y; medium; link not captured - search</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>